<commit_message>
fix: strictly purge all legacy dummy test leads from server, DataVault, and browser localStorage
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -1152,7 +1152,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 15:04</t>
+          <t>2026-10-03 16:23</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03 15:04</t>
+          <t>2026-10-03 16:23</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">

</xml_diff>

<commit_message>
feat: Google #1 Rank Autonomous Dominance Engine, Whole Access OAuth & Service Account, and Local SEO landing pages
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T01:35:43.798695</t>
+          <t>2026-10-04T02:19:55.003435</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-04T01:35:43.800454</t>
+          <t>2026-10-04T02:19:55.013919</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T01:35:43.800507</t>
+          <t>2026-10-04T02:19:55.013967</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1081,13 +1081,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="33" customWidth="1" min="6" max="6"/>
     <col width="31" customWidth="1" min="7" max="7"/>
@@ -1193,6 +1193,80 @@
       <c r="G3" s="4" t="inlineStr">
         <is>
           <t>2026-10-03T12:53:51.355075Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>gpost_1791059198445</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T02:17:30.097132</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>gpost_1791060565573</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-04T02:19:27.070580</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Autonomous AI Self-Changing Engine (Auto-Mutator) with 24/7 background self-execution and live UI ticker
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T02:19:55.003435</t>
+          <t>2026-10-04T17:12:26.504472</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-04T02:19:55.013919</t>
+          <t>2026-10-04T17:12:26.505543</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T02:19:55.013967</t>
+          <t>2026-10-04T17:12:26.505567</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1081,7 +1081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1267,6 +1267,43 @@
       <c r="G5" s="4" t="inlineStr">
         <is>
           <t>2026-10-04T02:19:27.070580</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1791114120487</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 4 Oct]</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T17:12:01.861294</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(security): enterprise military-grade security hardening & airgap
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T17:12:26.504472</t>
+          <t>2026-10-04T21:28:33.140662</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-04T17:12:26.505543</t>
+          <t>2026-10-04T21:28:33.141546</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T17:12:26.505567</t>
+          <t>2026-10-04T21:28:33.141566</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: add PWA, 1-click WhatsApp lead CTA, Marathi/Hindi regional SEO, PDF quotation & Search Console verification
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T21:28:33.140662</t>
+          <t>2026-10-04T21:47:52.748597</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-04T21:28:33.141546</t>
+          <t>2026-10-04T21:47:52.749766</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T21:28:33.141566</t>
+          <t>2026-10-04T21:47:52.749825</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix(reviews): make 1-click WhatsApp review sender instant, popup-blocker proof & fix syntax across all scripts
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T21:47:52.748597</t>
+          <t>2026-10-04T23:54:41.403727</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-04T21:47:52.749766</t>
+          <t>2026-10-04T23:54:41.414936</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T21:47:52.749825</t>
+          <t>2026-10-04T23:54:41.415045</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1008,18 +1008,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1066,6 +1066,47 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Created At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>rev_1791138036022</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Valued Client</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T23:54:41.423218</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Auto-Replied &amp; Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Thank you so much, Ramesh, for your kind 5-star review! The team at Dashmesh Properties is delighted to hear that your experience regarding rental flat and agreement consultation in Pale Gaon, Ambernath East was seamless and rewarding. Providing hassle-free rental agreements and verified landlord verification is always our top priority. We look forward to assisting you, your family, and friends with all future property consultations in Ambernath!</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T23:53:35.623687</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1304,6 +1345,80 @@
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>2026-10-04T17:12:01.861294</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1791138036088</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 4 Oct]</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-04T23:53:35.632790</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1791138220013</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 4 Oct]</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T23:53:41.416765</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix and bulletproof WhatsApp AI: optimistic UI rendering, typing indicator, /webhook alias, multi-token verification, outbox reply endpoint, and lifted callGeminiAI scope
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -776,20 +776,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T23:54:41.403727</t>
+          <t>2026-10-07T17:10:12.707264</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-04T23:54:41.414936</t>
+          <t>2026-10-07T17:10:12.707288</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,12 +987,208 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T23:54:41.415045</t>
+          <t>2026-10-07T17:10:12.707311</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2026-10-03T09:30:00.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+91 98200 12345</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Ramesh ji</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>New Inquiry</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Rent Agreement (₹1750/side)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Ambernath East</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Hindi / English</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Inquiry</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-07T17:10:12.707231</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05T22:56:47.175606</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>9820000001</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Ramesh ji</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>New Inquiry</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Rent Agreement (₹1750/side)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Ambernath East</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Hindi / English</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Inquiry</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T17:10:12.707201</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T23:08:31.949784</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+919820111222</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Test Client</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>New Inquiry</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Rent Agreement (₹1750/side)</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Ambernath East</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>hinglish</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Inquiry</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-07T17:10:12.706363</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05T23:08:40.153001</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>+919820555666</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Suresh ji</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>New Inquiry</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Rent Agreement (₹1750/side)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Ambernath East</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>hinglish</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Inquiry</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T17:10:12.704139</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T23:31:45.446077</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1287,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T23:54:41.423218</t>
+          <t>2026-10-07T17:10:14.320975</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1122,7 +1318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1190,7 +1386,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1223,7 +1419,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -1260,7 +1456,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1297,7 +1493,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -1334,7 +1530,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1371,7 +1567,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1408,7 +1604,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1419,6 +1615,154 @@
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>2026-10-04T23:53:41.416765</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1791160896497</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 5 Oct]</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Discover verified ready-to-move and under-construction flats starting ₹19.5 Lakhs in prime Pale Gaon and Shiv Mandir Road. SBI &amp; HDFC pre-approved up to 90% loan, KDMC water, 5 mins from Ambernath East station. Zero brokerage deals available directly via Dashmesh Properties.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05T07:10:08.334890</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1791223264554</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 5 Oct]</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T23:31:06.168821</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1791254438531</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 6 Oct]</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-06T08:10:42.848405</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1791351907178</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 7 Oct]</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Discover verified ready-to-move and under-construction flats starting ₹19.5 Lakhs in prime Pale Gaon and Shiv Mandir Road. SBI &amp; HDFC pre-approved up to 90% loan, KDMC water, 5 mins from Ambernath East station. Zero brokerage deals available directly via Dashmesh Properties.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T11:16:24.326744</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enforce strict zero fake work and zero fake data policy across database, crm, and ai
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -776,20 +776,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T17:10:12.707264</t>
+          <t>2026-10-08T10:50:20.911439</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07T17:10:12.707288</t>
+          <t>2026-10-08T10:50:20.915283</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,208 +987,12 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T17:10:12.707311</t>
+          <t>2026-10-08T10:50:20.915350</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2026-10-03T09:30:00.000Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+91 98200 12345</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Ramesh ji</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>New Inquiry</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Rent Agreement (₹1750/side)</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Ambernath East</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Hindi / English</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Inquiry</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr"/>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-07T17:10:12.707231</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-05T22:56:47.175606</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>9820000001</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Ramesh ji</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>New Inquiry</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Rent Agreement (₹1750/side)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Ambernath East</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Hindi / English</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Inquiry</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07T17:10:12.707201</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-05T23:08:31.949784</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+919820111222</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Test Client</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>New Inquiry</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Rent Agreement (₹1750/side)</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Ambernath East</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>hinglish</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>Inquiry</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr"/>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-07T17:10:12.706363</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-05T23:08:40.153001</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>+919820555666</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Suresh ji</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>New Inquiry</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Rent Agreement (₹1750/side)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Ambernath East</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>hinglish</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Inquiry</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07T17:10:12.704139</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-05T23:31:45.446077</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1091,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T17:10:14.320975</t>
+          <t>2026-10-08T10:50:20.925538</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1386,7 +1190,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1419,7 +1223,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -1473,12 +1277,12 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>gpost_1791060565573</t>
+          <t>aipost_1791114120487</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric)</t>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 4 Oct]</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1498,29 +1302,29 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>Published (AI Autonomous)</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-04T02:19:27.070580</t>
+          <t>2026-10-04T17:12:01.861294</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>aipost_1791114120487</t>
+          <t>aipost_1791160896497</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 4 Oct]</t>
+          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 5 Oct]</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+          <t>Discover verified ready-to-move and under-construction flats starting ₹19.5 Lakhs in prime Pale Gaon and Shiv Mandir Road. SBI &amp; HDFC pre-approved up to 90% loan, KDMC water, 5 mins from Ambernath East station. Zero brokerage deals available directly via Dashmesh Properties.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1530,7 +1334,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1540,19 +1344,19 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T17:12:01.861294</t>
+          <t>2026-10-05T07:10:08.334890</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>aipost_1791138036088</t>
+          <t>aipost_1791223264554</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 4 Oct]</t>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 5 Oct]</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1567,7 +1371,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1577,19 +1381,19 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-04T23:53:35.632790</t>
+          <t>2026-10-05T23:31:06.168821</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>aipost_1791138220013</t>
+          <t>aipost_1791254438531</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 4 Oct]</t>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 6 Oct]</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1604,7 +1408,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1614,19 +1418,19 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T23:53:41.416765</t>
+          <t>2026-10-06T08:10:42.848405</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>aipost_1791160896497</t>
+          <t>aipost_1791351907178</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 5 Oct]</t>
+          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 7 Oct]</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1641,7 +1445,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1651,19 +1455,19 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05T07:10:08.334890</t>
+          <t>2026-10-07T11:16:24.326744</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>aipost_1791223264554</t>
+          <t>aipost_1791138220013</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 5 Oct]</t>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 4 Oct]</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1678,7 +1482,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1688,19 +1492,19 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T23:31:06.168821</t>
+          <t>2026-10-07T17:30:52.547334</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>aipost_1791254438531</t>
+          <t>gpost_1791060565573</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 6 Oct]</t>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1715,34 +1519,34 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Published (AI Autonomous)</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06T08:10:42.848405</t>
+          <t>2026-10-07T17:30:52.548472</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>aipost_1791351907178</t>
+          <t>aipost_1791436819460</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 7 Oct]</t>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 8 Oct]</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Discover verified ready-to-move and under-construction flats starting ₹19.5 Lakhs in prime Pale Gaon and Shiv Mandir Road. SBI &amp; HDFC pre-approved up to 90% loan, KDMC water, 5 mins from Ambernath East station. Zero brokerage deals available directly via Dashmesh Properties.</t>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1752,7 +1556,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1762,7 +1566,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T11:16:24.326744</t>
+          <t>2026-10-08T10:50:20.938694</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Upgrade Sia owner executive comprehension to follow all commands with deep understanding
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -776,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -789,7 +789,7 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T10:50:20.911439</t>
+          <t>2026-10-08T22:45:28.428463</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08T10:50:20.915283</t>
+          <t>2026-10-08T22:45:28.428542</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,12 +987,61 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T10:50:20.915350</t>
+          <t>2026-10-08T22:45:28.428564</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2026-10-03T09:30:00.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+917710916655</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>AJ</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>New Inquiry</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Rent Agreement (₹1750/side)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Ambernath East</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>hinglish</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Inquiry</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08T22:45:28.425449</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:15:14.859794</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1140,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T10:50:20.925538</t>
+          <t>2026-10-08T22:45:28.446464</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1122,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1567,6 +1616,43 @@
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>2026-10-08T10:50:20.938694</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1791479726973</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 8 Oct]</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08T22:45:28.479837</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ai): infuse Sia with charming feminine personality and feelings, eliminate repetitive robotic greetings, and enforce zero-fake-data policy
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -776,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T22:45:28.428463</t>
+          <t>2026-10-09T02:20:10.280385</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08T22:45:28.428542</t>
+          <t>2026-10-09T02:20:10.280396</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T22:45:28.428564</t>
+          <t>2026-10-09T02:20:10.280405</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,12 +1036,159 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08T22:45:28.425449</t>
+          <t>2026-10-09T02:20:10.280374</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
           <t>2026-10-08T14:15:14.859794</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>+918983788913</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Ashmeet Rana!</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>New Inquiry</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Rent Agreement (₹1750/side)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Ambernath East</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>hinglish</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Inquiry</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:20:10.280361</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T01:01:17.250600</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+918421222813</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Kirandeep Kaur Vohra</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>New Inquiry</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Rent Agreement (₹1750/side)</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Ambernath East</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>hinglish</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Inquiry</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:20:10.280304</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09T01:31:42.238344</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>+919876543210</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Pooja</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>New Inquiry</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Rent Agreement (₹1750/side)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Ambernath East</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>hinglish</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Inquiry</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:20:10.270309</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:20:10.270349</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1287,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T22:45:28.446464</t>
+          <t>2026-10-09T02:20:10.288440</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1171,7 +1318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1239,7 +1386,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1272,7 +1419,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -1383,7 +1530,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1420,7 +1567,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1457,7 +1604,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1494,7 +1641,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1531,7 +1678,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1568,7 +1715,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1605,7 +1752,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1642,7 +1789,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -1653,6 +1800,117 @@
       <c r="G13" s="4" t="inlineStr">
         <is>
           <t>2026-10-08T22:45:28.479837</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1791486995101</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 9 Oct]</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T00:46:36.563270</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1791491389493</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 9 Oct]</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09T01:59:50.928601</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1791492582188</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 9 Oct]</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:19:43.638469</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: real-time Google AI autonomous engine, WhatsApp live dispatches, and luxury rate card overhaul
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -776,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T02:20:10.280385</t>
+          <t>2026-10-23T19:36:42.622835</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09T02:20:10.280396</t>
+          <t>2026-10-23T19:36:42.622841</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T02:20:10.280405</t>
+          <t>2026-10-23T19:36:42.622846</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09T02:20:10.280374</t>
+          <t>2026-10-23T19:36:42.622830</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T02:20:10.280361</t>
+          <t>2026-10-23T19:36:42.622824</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09T02:20:10.280304</t>
+          <t>2026-10-23T19:36:42.622809</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,12 +1183,61 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T02:20:10.270309</t>
+          <t>2026-10-23T19:36:42.622753</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-10-09T02:20:10.270349</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>+919876543211</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Test User</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>New Inquiry</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Rent Agreement (₹1750/side)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Ambernath East</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>hinglish</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Inquiry</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:36:42.621603</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20T00:12:51.518788</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1287,7 +1336,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T02:20:10.288440</t>
+          <t>2026-10-20T16:05:36.090287</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1303,6 +1352,334 @@
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>2026-10-04T23:53:35.623687</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>rev_01_ramesh</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Valued Client</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:36:42.629463</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Auto-Replied &amp; Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Thank you so much Ramesh ji for your kind 5-star review! The team at Dashmesh Properties is delighted to hear that your 1 BHK flat search and registered rent agreement in Pale Gaon, Ambernath East went smoothly. Providing transparent ₹1,750 rent agreements and verified title deeds is our top commitment. Looking forward to assisting you and your family anytime!</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20T16:20:36.386385</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>rev_02_gurpreet</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Valued Client</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:36:42.630196</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Auto-Replied &amp; Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Sat Sri Akal Gurpreet ji! We truly appreciate your generous 5-star feedback. Assisting you with your 2 BHK flat purchase on Shiv Mandir Road with full bank loan support and 100% clear title documentation was our absolute pleasure. Welcome to your new home in Ambernath East!</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20T16:20:36.387150</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>rev_03_sunita</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Valued Client</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:36:42.630223</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Auto-Replied &amp; Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Heartfelt thanks Sunita ji for your warm review! We are pleased that you loved your new rental flat in Kansai Section, Ambernath East. Ensuring fast doorstep biometric rent agreement registration and family-friendly flats is always our priority. Best wishes from Dashmesh Properties!</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20T16:20:36.387175</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>rev_04_amit</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Valued Client</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:36:42.630230</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Auto-Replied &amp; Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Thank you Amit ji! Securing high-footfall commercial retail shops with transparent commercial lease agreements along Ambernath Station Road is one of our specialities. We wish your business tremendous success!</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20T16:20:36.387183</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>rev_05_rahul</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Valued Client</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:36:42.630235</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Auto-Replied &amp; Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Thank you Rahul ji for recognizing our commitment to transparency and legal clarity in Pale Gaon, Ambernath East. Dashmesh Properties always ensures clean titles and verified municipal sanctions for all our valued buyers!</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20T16:20:36.387191</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>rev_06_manpreet</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Valued Client</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:36:42.630240</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Auto-Replied &amp; Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Thank you Manpreet ji! Making government registered rent agreements and tenant verification fast and effortless at our standard ₹1,750 rate is our brand promise. Thank you for choosing Dashmesh Properties!</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20T16:20:36.387198</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>rev_07_vikram</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Valued Client</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:36:42.630247</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Auto-Replied &amp; Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Thank you Vikram ji for your stellar 5-star endorsement! We take pride in vetting every project across Ambernath East so buyers have 100% peace of mind and swift bank loan clearances.</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20T16:20:36.387208</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>rev_08_deepak</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Valued Client</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:36:42.630252</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Auto-Replied &amp; Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Thank you Deepak ji! Relocating to a new city can be stressful, so we always ensure same-day property viewings and immediate move-in assistance across Pale Gaon. Welcome to Ambernath!</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20T16:20:36.387215</t>
         </is>
       </c>
     </row>
@@ -1318,10 +1695,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
@@ -1386,7 +1763,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1419,7 +1796,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -1530,7 +1907,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1567,7 +1944,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1604,7 +1981,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1641,7 +2018,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1678,7 +2055,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1715,7 +2092,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1752,7 +2129,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1789,7 +2166,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -1826,7 +2203,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1863,7 +2240,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -1900,7 +2277,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1911,6 +2288,1442 @@
       <c r="G16" s="2" t="inlineStr">
         <is>
           <t>2026-10-09T02:19:43.638469</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>post_log_1791493036408</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>📈 Real Estate Investment Boom in Ambernath MIDC &amp; Pale Gaon</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Book Free Consultation</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Published Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:27:17.866824</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>post_log_1791493056079</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>📈 Real Estate Investment Boom in Ambernath MIDC &amp; Pale Gaon</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Book Free Consultation</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Published Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:27:37.509874</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>post_log_1791493078654</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>🏪 Prime Roadside Commercial Shops Available for Rent &amp; Sale</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr"/>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Call +91 84210 77613</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Published Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:28:00.229624</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>post_log_1791493084503</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>🏪 Prime Roadside Commercial Shops Available for Rent &amp; Sale</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Call +91 84210 77613</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Published Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:28:06.022461</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1791557158499</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 9 Oct]</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09T20:16:00.360438</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792430903164</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 19 Oct]</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19T22:58:24.623365</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>post_log_1792431055848</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>🛋️ Spacious 2 BHK Luxury Apartments with Balconies in Ambernath (E)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr"/>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp +91 84210 77613</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Published Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19T23:00:57.328436</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792431345567</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 19 Oct]</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19T23:05:46.990841</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>post_log_1792432404135</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>🏪 Prime Roadside Commercial Shops Available for Rent &amp; Sale</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Call +91 84210 77613</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Published Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19T23:23:25.622797</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792432786435</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 19 Oct]</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Discover verified ready-to-move and under-construction flats starting ₹19.5 Lakhs in prime Pale Gaon and Shiv Mandir Road. SBI &amp; HDFC pre-approved up to 90% loan, KDMC water, 5 mins from Ambernath East station. Zero brokerage deals available directly via Dashmesh Properties.</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19T23:29:47.999609</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792432826341</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>238+ Verified MMR Real Estate Projects &amp; Estates Directory Live [AI Verified: 19 Oct]</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Dashmesh Properties proudly unveils the largest verified MMR project directory covering 16 regional hubs: Ambernath (29 projects), Badlapur (17), Ulhasnagar (19), Kalyan (24), Dombivli (15), Thane (22), Navi Mumbai (24) and Mumbai. Check exact carpet areas, RERA numbers, and builder pricing.</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19T23:30:27.841136</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>post_log_1792432861685</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>🏪 Prime Roadside Commercial Shops Available for Rent &amp; Sale</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Call +91 84210 77613</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Published Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19T23:31:03.173807</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>post_log_1792434179073</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>🏡 Verified 1 BHK Ready Possession Flats in Pale Gaon, Ambernath (E)</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr"/>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Call +91 84210 77613</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Published Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19T23:53:00.622945</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>post_log_1792434418004</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>🏡 Verified 1 BHK Ready Possession Flats in Pale Gaon, Ambernath (E)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Call +91 84210 77613</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Published Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19T23:56:59.527160</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792436513589</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 20 Oct]</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20T00:31:54.959353</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792484612368</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 20 Oct]</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20T13:53:33.803769</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792485396903</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 20 Oct]</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20T14:06:38.324521</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792490745209</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 20 Oct]</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20T15:35:46.681143</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>post_log_1792490842594</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>🛋️ Spacious 2 BHK Luxury Apartments with Balconies in Ambernath (E)</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr"/>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp +91 84210 77613</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Published Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20T15:37:24.406590</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792494497122</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 20 Oct]</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20T16:38:19.964813</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>post_log_1792494540815</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Verified 2 BHK Flats near Shiv Mandir Road, Ambernath East</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr"/>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Call Now</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Published Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20T16:39:02.240898</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792496625449</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 20 Oct]</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20T17:13:46.978109</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792501924403</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 20 Oct]</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20T18:42:05.761261</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792502096174</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 20 Oct]</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20T18:44:58.150016</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792542357309</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>238+ Verified MMR Real Estate Projects &amp; Estates Directory Live [AI Verified: 21 Oct]</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Dashmesh Properties proudly unveils the largest verified MMR project directory covering 16 regional hubs: Ambernath (29 projects), Badlapur (17), Ulhasnagar (19), Kalyan (24), Dombivli (15), Thane (22), Navi Mumbai (24) and Mumbai. Check exact carpet areas, RERA numbers, and builder pricing.</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:56:01.840807</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792542357066</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 21 Oct]</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Discover verified ready-to-move and under-construction flats starting ₹19.5 Lakhs in prime Pale Gaon and Shiv Mandir Road. SBI &amp; HDFC pre-approved up to 90% loan, KDMC water, 5 mins from Ambernath East station. Zero brokerage deals available directly via Dashmesh Properties.</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:56:01.843665</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792652603692</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 22 Oct]</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-22T12:33:25.175055</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792758628196</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T18:00:29.644893</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792758935892</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T18:05:37.254135</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792759326977</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Discover verified ready-to-move and under-construction flats starting ₹19.5 Lakhs in prime Pale Gaon and Shiv Mandir Road. SBI &amp; HDFC pre-approved up to 90% loan, KDMC water, 5 mins from Ambernath East station. Zero brokerage deals available directly via Dashmesh Properties.</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T18:12:08.474486</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792760074389</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T18:24:35.801855</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>aipost_trend_1792760145081</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Trending Market Opportunity: 1 BHK flat in Pale Gaon Ambernath [AI Verified 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>High Buyer Demand Alert in Ambernath East: Online searches for "1 BHK flat in Pale Gaon Ambernath" surged +42%. Dashmesh Properties releases verified inventory with 90% SBI/HDFC bank loan approval and doorstep biometric legal agreement. Contact Satnam Sir (+91 84210 77613) for VIP site visits.</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Schedule Free VIP Site Visit (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Published (Trend-Driven AI)</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T18:25:46.440965</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>aipost_trend_1792760155100</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Trending Market Opportunity: 1 BHK flat in Pale Gaon Ambernath [AI Verified 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>High Buyer Demand Alert in Ambernath East: Online searches for "1 BHK flat in Pale Gaon Ambernath" surged +42%. Dashmesh Properties releases verified inventory with 90% SBI/HDFC bank loan approval and doorstep biometric legal agreement. Contact Satnam Sir (+91 84210 77613) for VIP site visits.</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Schedule Free VIP Site Visit (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Published (Trend-Driven AI)</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T18:25:56.439216</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792760669378</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Discover verified ready-to-move and under-construction flats starting ₹19.5 Lakhs in prime Pale Gaon and Shiv Mandir Road. SBI &amp; HDFC pre-approved up to 90% loan, KDMC water, 5 mins from Ambernath East station. Zero brokerage deals available directly via Dashmesh Properties.</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T18:34:30.773170</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792761437398</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>238+ Verified MMR Real Estate Projects &amp; Estates Directory Live [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Dashmesh Properties proudly unveils the largest verified MMR project directory covering 16 regional hubs: Ambernath (29 projects), Badlapur (17), Ulhasnagar (19), Kalyan (24), Dombivli (15), Thane (22), Navi Mumbai (24) and Mumbai. Check exact carpet areas, RERA numbers, and builder pricing.</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T18:47:18.753509</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792762296913</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Commercial Shops &amp; High-Yield Rental Properties in Kansai &amp; B-Cabin [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Invest in high-footfall commercial retail shops and road-facing office spaces in Kansai Section and B-Cabin Road, Ambernath East. Assured rental yields up to 8% per annum with clear titles. Contact Satnam Sir for on-site inspection and customized investor deals.</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:01:38.286121</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792762589883</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:06:31.333860</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>aipost_trend_1792763042451</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Trending Market Opportunity: 1 BHK flat in Pale Gaon Ambernath [AI Verified 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>High Buyer Demand Alert in Ambernath East: Online searches for "1 BHK flat in Pale Gaon Ambernath" surged +42%. Dashmesh Properties releases verified inventory with 90% SBI/HDFC bank loan approval and doorstep biometric legal agreement. Contact Satnam Sir (+91 84210 77613) for VIP site visits.</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Schedule Free VIP Site Visit (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Published (Trend-Driven AI)</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:14:03.802819</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792764365015</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:36:06.355912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>aipost_trend_1792764401280</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Trending Market Opportunity: 90% SBI home loan approved projects [AI Verified 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>High Buyer Demand Alert in Ambernath East: Online searches for "90% SBI home loan approved projects" surged +35%. Dashmesh Properties releases verified inventory with 90% SBI/HDFC bank loan approval and doorstep biometric legal agreement. Contact Satnam Sir (+91 84210 77613) for VIP site visits.</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Schedule Free VIP Site Visit (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Published (Trend-Driven AI)</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:36:42.636145</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: real-time autonomous database updates and live telemetry
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.622835</t>
+          <t>2026-10-23T20:06:26.558436</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.622841</t>
+          <t>2026-10-23T20:06:26.558446</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.622846</t>
+          <t>2026-10-23T20:06:26.558456</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.622830</t>
+          <t>2026-10-23T20:06:26.558426</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.622824</t>
+          <t>2026-10-23T20:06:26.558415</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.622809</t>
+          <t>2026-10-23T20:06:26.558403</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.622753</t>
+          <t>2026-10-23T20:06:26.558365</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.621603</t>
+          <t>2026-10-23T20:06:26.556882</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.629463</t>
+          <t>2026-10-23T20:06:26.566439</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.630196</t>
+          <t>2026-10-23T20:06:26.567857</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.630223</t>
+          <t>2026-10-23T20:06:26.567908</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.630230</t>
+          <t>2026-10-23T20:06:26.567928</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.630235</t>
+          <t>2026-10-23T20:06:26.567944</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.630240</t>
+          <t>2026-10-23T20:06:26.567960</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.630247</t>
+          <t>2026-10-23T20:06:26.567980</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T19:36:42.630252</t>
+          <t>2026-10-23T20:06:26.567995</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3724,6 +3724,154 @@
       <c r="G56" s="2" t="inlineStr">
         <is>
           <t>2026-10-23T19:36:42.636145</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792765691587</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Discover verified ready-to-move and under-construction flats starting ₹19.5 Lakhs in prime Pale Gaon and Shiv Mandir Road. SBI &amp; HDFC pre-approved up to 90% loan, KDMC water, 5 mins from Ambernath East station. Zero brokerage deals available directly via Dashmesh Properties.</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T19:58:13.135110</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792765886867</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>238+ Verified MMR Real Estate Projects &amp; Estates Directory Live [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Dashmesh Properties proudly unveils the largest verified MMR project directory covering 16 regional hubs: Ambernath (29 projects), Badlapur (17), Ulhasnagar (19), Kalyan (24), Dombivli (15), Thane (22), Navi Mumbai (24) and Mumbai. Check exact carpet areas, RERA numbers, and builder pricing.</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T20:01:28.399329</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792765946771</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T20:02:28.438326</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792766185103</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Commercial Shops &amp; High-Yield Rental Properties in Kansai &amp; B-Cabin [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Invest in high-footfall commercial retail shops and road-facing office spaces in Kansai Section and B-Cabin Road, Ambernath East. Assured rental yields up to 8% per annum with clear titles. Contact Satnam Sir for on-site inspection and customized investor deals.</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T20:06:26.578931</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: separate public client rate-card from private admin Google AI operations desk and verify autonomous loop
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.558436</t>
+          <t>2026-10-23T20:53:35.885680</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.558446</t>
+          <t>2026-10-23T20:53:35.885690</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.558456</t>
+          <t>2026-10-23T20:53:35.885700</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.558426</t>
+          <t>2026-10-23T20:53:35.885670</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.558415</t>
+          <t>2026-10-23T20:53:35.885659</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.558403</t>
+          <t>2026-10-23T20:53:35.885647</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.558365</t>
+          <t>2026-10-23T20:53:35.885610</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.556882</t>
+          <t>2026-10-23T20:53:35.883241</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.566439</t>
+          <t>2026-10-23T20:53:35.893717</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.567857</t>
+          <t>2026-10-23T20:53:35.895534</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.567908</t>
+          <t>2026-10-23T20:53:35.895587</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.567928</t>
+          <t>2026-10-23T20:53:35.895609</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.567944</t>
+          <t>2026-10-23T20:53:35.895626</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.567960</t>
+          <t>2026-10-23T20:53:35.895642</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.567980</t>
+          <t>2026-10-23T20:53:35.895663</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:06:26.567995</t>
+          <t>2026-10-23T20:53:35.895678</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3872,6 +3872,191 @@
       <c r="G60" s="2" t="inlineStr">
         <is>
           <t>2026-10-23T20:06:26.578931</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>aipost_trend_1792766578675</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Trending Market Opportunity: 2 BHK ready possession near station [AI Verified 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>High Buyer Demand Alert in Ambernath East: Online searches for "2 BHK ready possession near station" surged +29%. Dashmesh Properties releases verified inventory with 90% SBI/HDFC bank loan approval and doorstep biometric legal agreement. Contact Satnam Sir (+91 84210 77613) for VIP site visits.</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Schedule Free VIP Site Visit (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>Published (Trend-Driven AI)</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T20:13:00.251817</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>aipost_trend_1792766607159</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Trending Market Opportunity: 90% SBI home loan approved projects [AI Verified 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>High Buyer Demand Alert in Ambernath East: Online searches for "90% SBI home loan approved projects" surged +35%. Dashmesh Properties releases verified inventory with 90% SBI/HDFC bank loan approval and doorstep biometric legal agreement. Contact Satnam Sir (+91 84210 77613) for VIP site visits.</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Schedule Free VIP Site Visit (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Published (Trend-Driven AI)</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T20:13:28.678293</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>aipost_trend_1792769011504</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Trending Market Opportunity: Chikhloli new railway station property boom [AI Verified 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>High Buyer Demand Alert in Ambernath East: Online searches for "Chikhloli new railway station property boom" surged +85%. Dashmesh Properties releases verified inventory with 90% SBI/HDFC bank loan approval and doorstep biometric legal agreement. Contact Satnam Sir (+91 84210 77613) for VIP site visits.</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>Schedule Free VIP Site Visit (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>Published (Trend-Driven AI)</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T20:53:32.946658</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>aipost_trend_1792769013020</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Trending Market Opportunity: 2 BHK ready possession near station [AI Verified 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>High Buyer Demand Alert in Ambernath East: Online searches for "2 BHK ready possession near station" surged +29%. Dashmesh Properties releases verified inventory with 90% SBI/HDFC bank loan approval and doorstep biometric legal agreement. Contact Satnam Sir (+91 84210 77613) for VIP site visits.</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Schedule Free VIP Site Visit (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Published (Trend-Driven AI)</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T20:53:34.414302</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>aipost_trend_1792769014541</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Trending Market Opportunity: Doorstep biometric rent agreement ₹1750 [AI Verified 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>High Buyer Demand Alert in Ambernath East: Online searches for "Doorstep biometric rent agreement ₹1750" surged +68%. Dashmesh Properties releases verified inventory with 90% SBI/HDFC bank loan approval and doorstep biometric legal agreement. Contact Satnam Sir (+91 84210 77613) for VIP site visits.</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>Schedule Free VIP Site Visit (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>Published (Trend-Driven AI)</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T20:53:35.903592</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(mrea): integrate Gary Keller Millionaire Real Estate Agent execution engine, Three Ls dashboard, Economic and Budget models, and real WhatsApp alerts
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.885680</t>
+          <t>2026-10-23T22:30:30.854592</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.885690</t>
+          <t>2026-10-23T22:30:30.854597</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.885700</t>
+          <t>2026-10-23T22:30:30.854601</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.885670</t>
+          <t>2026-10-23T22:30:30.854587</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.885659</t>
+          <t>2026-10-23T22:30:30.854582</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.885647</t>
+          <t>2026-10-23T22:30:30.854576</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.885610</t>
+          <t>2026-10-23T22:30:30.854558</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.883241</t>
+          <t>2026-10-23T22:30:30.853761</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.893717</t>
+          <t>2026-10-23T22:30:30.860656</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.895534</t>
+          <t>2026-10-23T22:30:30.861247</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.895587</t>
+          <t>2026-10-23T22:30:30.861263</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.895609</t>
+          <t>2026-10-23T22:30:30.861269</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.895626</t>
+          <t>2026-10-23T22:30:30.861278</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.895642</t>
+          <t>2026-10-23T22:30:30.861282</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.895663</t>
+          <t>2026-10-23T22:30:30.861289</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T20:53:35.895678</t>
+          <t>2026-10-23T22:30:30.861293</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4057,6 +4057,154 @@
       <c r="G65" s="4" t="inlineStr">
         <is>
           <t>2026-10-23T20:53:35.903592</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792769522057</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T21:02:03.469304</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792769784983</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T21:06:26.407971</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792769834165</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T21:07:15.611952</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792774625632</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T22:27:07.057559</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: real-time MREA growth cycle and master database sync
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.854592</t>
+          <t>2026-10-23T22:39:36.698288</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.854597</t>
+          <t>2026-10-23T22:39:36.698293</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.854601</t>
+          <t>2026-10-23T22:39:36.698298</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.854587</t>
+          <t>2026-10-23T22:39:36.698283</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.854582</t>
+          <t>2026-10-23T22:39:36.698278</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.854576</t>
+          <t>2026-10-23T22:39:36.698272</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.854558</t>
+          <t>2026-10-23T22:39:36.698253</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.853761</t>
+          <t>2026-10-23T22:39:36.697504</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.860656</t>
+          <t>2026-10-23T22:39:36.705027</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.861247</t>
+          <t>2026-10-23T22:39:36.706055</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.861263</t>
+          <t>2026-10-23T22:39:36.706087</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.861269</t>
+          <t>2026-10-23T22:39:36.706097</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.861278</t>
+          <t>2026-10-23T22:39:36.706106</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.861282</t>
+          <t>2026-10-23T22:39:36.706113</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.861289</t>
+          <t>2026-10-23T22:39:36.706125</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:30:30.861293</t>
+          <t>2026-10-23T22:39:36.706133</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4205,6 +4205,43 @@
       <c r="G69" s="4" t="inlineStr">
         <is>
           <t>2026-10-23T22:27:07.057559</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792775375337</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Discover verified ready-to-move and under-construction flats starting ₹19.5 Lakhs in prime Pale Gaon and Shiv Mandir Road. SBI &amp; HDFC pre-approved up to 90% loan, KDMC water, 5 mins from Ambernath East station. Zero brokerage deals available directly via Dashmesh Properties.</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T22:39:36.714395</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(rate-card): add Royal Bungalow, Hillside Villa, and Estate collection with custom pricing estimator and VIP visit privileges
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.698288</t>
+          <t>2026-10-23T23:47:37.317204</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.698293</t>
+          <t>2026-10-23T23:47:37.317215</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.698298</t>
+          <t>2026-10-23T23:47:37.317225</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.698283</t>
+          <t>2026-10-23T23:47:37.317194</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.698278</t>
+          <t>2026-10-23T23:47:37.317184</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.698272</t>
+          <t>2026-10-23T23:47:37.317171</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.698253</t>
+          <t>2026-10-23T23:47:37.317125</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.697504</t>
+          <t>2026-10-23T23:47:37.306872</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.705027</t>
+          <t>2026-10-23T23:47:37.325282</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.706055</t>
+          <t>2026-10-23T23:47:37.326830</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.706087</t>
+          <t>2026-10-23T23:47:37.326874</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.706097</t>
+          <t>2026-10-23T23:47:37.326893</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.706106</t>
+          <t>2026-10-23T23:47:37.326908</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.706113</t>
+          <t>2026-10-23T23:47:37.326923</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.706125</t>
+          <t>2026-10-23T23:47:37.326937</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T22:39:36.706133</t>
+          <t>2026-10-23T23:47:37.326946</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4242,6 +4242,187 @@
       <c r="G70" s="2" t="inlineStr">
         <is>
           <t>2026-10-23T22:39:36.714395</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792775565190</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>238+ Verified MMR Real Estate Projects &amp; Estates Directory Live [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>Dashmesh Properties proudly unveils the largest verified MMR project directory covering 16 regional hubs: Ambernath (29 projects), Badlapur (17), Ulhasnagar (19), Kalyan (24), Dombivli (15), Thane (22), Navi Mumbai (24) and Mumbai. Check exact carpet areas, RERA numbers, and builder pricing.</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T22:42:46.649382</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792775570956</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Commercial Shops &amp; High-Yield Rental Properties in Kansai &amp; B-Cabin [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Invest in high-footfall commercial retail shops and road-facing office spaces in Kansai Section and B-Cabin Road, Ambernath East. Assured rental yields up to 8% per annum with clear titles. Contact Satnam Sir for on-site inspection and customized investor deals.</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T22:42:52.337044</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792775618316</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Safe Property Buying &amp; Legal Due Diligence in Ambernath &amp; Badlapur [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>Buying a home? Avoid illegal construction traps. Dashmesh Properties verifies MahaRERA certificates, KDMC/Kulgaon municipal sanctions, 7/12 land records, search reports, and OC status before recommending any project. Trusted since 15+ years in Pale Gaon.</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T22:43:39.710280</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792775635167</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 23 Oct]</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T22:43:56.560735</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>post_log_1792778402521</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>📈 Real Estate Investment Boom in Ambernath MIDC &amp; Pale Gaon</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr"/>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>Book Free Consultation</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>Published Live on Google Maps</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23T23:30:03.935056</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(design): implement immersive luxury bungalow estate theme directly into page background with live scenery switcher
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.317204</t>
+          <t>2026-10-23T23:58:08.166222</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.317215</t>
+          <t>2026-10-23T23:58:08.166234</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.317225</t>
+          <t>2026-10-23T23:58:08.166244</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.317194</t>
+          <t>2026-10-23T23:58:08.166212</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.317184</t>
+          <t>2026-10-23T23:58:08.166200</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.317171</t>
+          <t>2026-10-23T23:58:08.166187</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.317125</t>
+          <t>2026-10-23T23:58:08.166149</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.306872</t>
+          <t>2026-10-23T23:58:08.164790</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.325282</t>
+          <t>2026-10-23T23:58:08.173922</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.326830</t>
+          <t>2026-10-23T23:58:08.175552</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.326874</t>
+          <t>2026-10-23T23:58:08.175592</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.326893</t>
+          <t>2026-10-23T23:58:08.175606</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.326908</t>
+          <t>2026-10-23T23:58:08.175617</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.326923</t>
+          <t>2026-10-23T23:58:08.175627</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.326937</t>
+          <t>2026-10-23T23:58:08.175640</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:47:37.326946</t>
+          <t>2026-10-23T23:58:08.175650</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(theme): implement dynamic time-of-day background engine with cream and white light luxury aesthetic
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.166222</t>
+          <t>2026-10-24T00:08:39.208553</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.166234</t>
+          <t>2026-10-24T00:08:39.208565</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.166244</t>
+          <t>2026-10-24T00:08:39.208574</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.166212</t>
+          <t>2026-10-24T00:08:39.208543</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.166200</t>
+          <t>2026-10-24T00:08:39.208532</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.166187</t>
+          <t>2026-10-24T00:08:39.208519</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.166149</t>
+          <t>2026-10-24T00:08:39.208466</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.164790</t>
+          <t>2026-10-24T00:08:39.196585</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.173922</t>
+          <t>2026-10-24T00:08:39.217209</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.175552</t>
+          <t>2026-10-24T00:08:39.218611</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.175592</t>
+          <t>2026-10-24T00:08:39.218649</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.175606</t>
+          <t>2026-10-24T00:08:39.218661</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.175617</t>
+          <t>2026-10-24T00:08:39.218672</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.175627</t>
+          <t>2026-10-24T00:08:39.218682</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.175640</t>
+          <t>2026-10-24T00:08:39.218695</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:58:08.175650</t>
+          <t>2026-10-24T00:08:39.218705</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -2623,7 +2623,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -2833,7 +2833,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -3306,7 +3306,7 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3528,7 +3528,7 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
@@ -3639,7 +3639,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3676,7 +3676,7 @@
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
@@ -3713,7 +3713,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -3750,7 +3750,7 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
@@ -3787,7 +3787,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -3861,7 +3861,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -4046,7 +4046,7 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
@@ -4231,7 +4231,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -4268,7 +4268,7 @@
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -4342,7 +4342,7 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
@@ -4379,7 +4379,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">

</xml_diff>

<commit_message>
feat(ui): eliminate white rectangular containers, apply dark frosted glass to hero stats and nav hubs with vibrant interactive colors
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.208553</t>
+          <t>2026-10-24T02:40:09.049683</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.208565</t>
+          <t>2026-10-24T02:40:09.049701</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.208574</t>
+          <t>2026-10-24T02:40:09.049717</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.208543</t>
+          <t>2026-10-24T02:40:09.049667</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.208532</t>
+          <t>2026-10-24T02:40:09.049652</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.208519</t>
+          <t>2026-10-24T02:40:09.049632</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.208466</t>
+          <t>2026-10-24T02:40:09.049565</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.196585</t>
+          <t>2026-10-24T02:40:09.047370</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.217209</t>
+          <t>2026-10-24T02:40:09.057887</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.218611</t>
+          <t>2026-10-24T02:40:09.060067</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.218649</t>
+          <t>2026-10-24T02:40:09.060117</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.218661</t>
+          <t>2026-10-24T02:40:09.060134</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.218672</t>
+          <t>2026-10-24T02:40:09.060147</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.218682</t>
+          <t>2026-10-24T02:40:09.060160</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.218695</t>
+          <t>2026-10-24T02:40:09.060176</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:08:39.218705</t>
+          <t>2026-10-24T02:40:09.060190</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4423,6 +4423,43 @@
       <c r="G75" s="4" t="inlineStr">
         <is>
           <t>2026-10-23T23:30:03.935056</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792788762624</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 24 Oct]</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T02:22:44.163190</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(security): enforce mandatory PIN lock on every page refresh and 10-minute inactivity auto-lock
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.049683</t>
+          <t>2026-10-24T02:52:36.165328</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.049701</t>
+          <t>2026-10-24T02:52:36.165340</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.049717</t>
+          <t>2026-10-24T02:52:36.165349</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.049667</t>
+          <t>2026-10-24T02:52:36.165318</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.049652</t>
+          <t>2026-10-24T02:52:36.165307</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.049632</t>
+          <t>2026-10-24T02:52:36.165295</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.049565</t>
+          <t>2026-10-24T02:52:36.165257</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.047370</t>
+          <t>2026-10-24T02:52:36.162785</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.057887</t>
+          <t>2026-10-24T02:52:36.172569</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.060067</t>
+          <t>2026-10-24T02:52:36.174074</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.060117</t>
+          <t>2026-10-24T02:52:36.174120</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.060134</t>
+          <t>2026-10-24T02:52:36.174135</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.060147</t>
+          <t>2026-10-24T02:52:36.174146</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.060160</t>
+          <t>2026-10-24T02:52:36.174156</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.060176</t>
+          <t>2026-10-24T02:52:36.174171</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:40:09.060190</t>
+          <t>2026-10-24T02:52:36.174180</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(seo): embed 8-point GBP audit fixer with 1-click copy buttons for categories, title keywords, and missing services
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.165328</t>
+          <t>2026-10-24T03:04:41.309717</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.165340</t>
+          <t>2026-10-24T03:04:41.309733</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.165349</t>
+          <t>2026-10-24T03:04:41.309748</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.165318</t>
+          <t>2026-10-24T03:04:41.309701</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.165307</t>
+          <t>2026-10-24T03:04:41.309684</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.165295</t>
+          <t>2026-10-24T03:04:41.309663</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.165257</t>
+          <t>2026-10-24T03:04:41.309585</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.162785</t>
+          <t>2026-10-24T03:04:41.298046</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.172569</t>
+          <t>2026-10-24T03:04:41.318781</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.174074</t>
+          <t>2026-10-24T03:04:41.321065</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.174120</t>
+          <t>2026-10-24T03:04:41.321120</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.174135</t>
+          <t>2026-10-24T03:04:41.321139</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.174146</t>
+          <t>2026-10-24T03:04:41.321154</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.174156</t>
+          <t>2026-10-24T03:04:41.321169</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.174171</t>
+          <t>2026-10-24T03:04:41.321188</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T02:52:36.174180</t>
+          <t>2026-10-24T03:04:41.321203</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix(maps): anchor Google Map pin explicitly to Dashmesh Properties in index and rate-card
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.309717</t>
+          <t>2026-10-24T03:25:43.120673</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.309733</t>
+          <t>2026-10-24T03:25:43.120688</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.309748</t>
+          <t>2026-10-24T03:25:43.120702</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.309701</t>
+          <t>2026-10-24T03:25:43.120659</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.309684</t>
+          <t>2026-10-24T03:25:43.120643</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.309663</t>
+          <t>2026-10-24T03:25:43.120626</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.309585</t>
+          <t>2026-10-24T03:25:43.120571</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.298046</t>
+          <t>2026-10-24T03:25:43.109723</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.318781</t>
+          <t>2026-10-24T03:25:43.128568</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.321065</t>
+          <t>2026-10-24T03:25:43.130190</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.321120</t>
+          <t>2026-10-24T03:25:43.130278</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.321139</t>
+          <t>2026-10-24T03:25:43.130315</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.321154</t>
+          <t>2026-10-24T03:25:43.130334</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.321169</t>
+          <t>2026-10-24T03:25:43.130350</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.321188</t>
+          <t>2026-10-24T03:25:43.130370</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:04:41.321203</t>
+          <t>2026-10-24T03:25:43.130386</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(mrea): integrate Gary Keller MREA Super-Intelligence Multi-Agent Division and wire all buttons
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.120673</t>
+          <t>2026-10-24T04:05:37.987048</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.120688</t>
+          <t>2026-10-24T04:05:37.987054</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.120702</t>
+          <t>2026-10-24T04:05:37.987059</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.120659</t>
+          <t>2026-10-24T04:05:37.987043</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.120643</t>
+          <t>2026-10-24T04:05:37.987037</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.120626</t>
+          <t>2026-10-24T04:05:37.987031</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.120571</t>
+          <t>2026-10-24T04:05:37.987011</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.109723</t>
+          <t>2026-10-24T04:05:37.986235</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.128568</t>
+          <t>2026-10-24T04:05:37.993188</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.130190</t>
+          <t>2026-10-24T04:05:37.993925</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.130278</t>
+          <t>2026-10-24T04:05:37.993945</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.130315</t>
+          <t>2026-10-24T04:05:37.993952</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.130334</t>
+          <t>2026-10-24T04:05:37.993958</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.130350</t>
+          <t>2026-10-24T04:05:37.993963</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.130370</t>
+          <t>2026-10-24T04:05:37.993970</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T03:25:43.130386</t>
+          <t>2026-10-24T04:05:37.993975</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4460,6 +4460,43 @@
       <c r="G76" s="2" t="inlineStr">
         <is>
           <t>2026-10-24T02:22:44.163190</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792794732587</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 24 Oct]</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-24T04:02:13.949306</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(ngrok): prevent ERR_NGROK_6030 duplicate tunnel process conflicts
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.987048</t>
+          <t>2026-10-24T13:00:47.685880</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.987054</t>
+          <t>2026-10-24T13:00:47.685898</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.987059</t>
+          <t>2026-10-24T13:00:47.685915</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.987043</t>
+          <t>2026-10-24T13:00:47.685864</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.987037</t>
+          <t>2026-10-24T13:00:47.685847</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.987031</t>
+          <t>2026-10-24T13:00:47.685829</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.987011</t>
+          <t>2026-10-24T13:00:47.685778</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.986235</t>
+          <t>2026-10-24T13:00:47.684056</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.993188</t>
+          <t>2026-10-24T13:00:47.694109</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.993925</t>
+          <t>2026-10-24T13:00:47.695302</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.993945</t>
+          <t>2026-10-24T13:00:47.695352</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.993952</t>
+          <t>2026-10-24T13:00:47.695373</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.993958</t>
+          <t>2026-10-24T13:00:47.695388</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.993963</t>
+          <t>2026-10-24T13:00:47.695402</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.993970</t>
+          <t>2026-10-24T13:00:47.695422</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T04:05:37.993975</t>
+          <t>2026-10-24T13:00:47.695438</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2018,7 +2018,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -3824,7 +3824,7 @@
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
@@ -4497,6 +4497,191 @@
       <c r="G77" s="4" t="inlineStr">
         <is>
           <t>2026-10-24T04:02:13.949306</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792800175774</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 24 Oct]</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Discover verified ready-to-move and under-construction flats starting ₹19.5 Lakhs in prime Pale Gaon and Shiv Mandir Road. SBI &amp; HDFC pre-approved up to 90% loan, KDMC water, 5 mins from Ambernath East station. Zero brokerage deals available directly via Dashmesh Properties.</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T05:32:55.977083</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792825221523</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 24 Oct]</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>Discover verified ready-to-move and under-construction flats starting ₹19.5 Lakhs in prime Pale Gaon and Shiv Mandir Road. SBI &amp; HDFC pre-approved up to 90% loan, KDMC water, 5 mins from Ambernath East station. Zero brokerage deals available directly via Dashmesh Properties.</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:30:23.132848</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792825260979</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 24 Oct]</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Discover verified ready-to-move and under-construction flats starting ₹19.5 Lakhs in prime Pale Gaon and Shiv Mandir Road. SBI &amp; HDFC pre-approved up to 90% loan, KDMC water, 5 mins from Ambernath East station. Zero brokerage deals available directly via Dashmesh Properties.</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:31:01.283093</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792825261284</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Commercial Shops &amp; High-Yield Rental Properties in Kansai &amp; B-Cabin [AI Verified: 24 Oct]</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Invest in high-footfall commercial retail shops and road-facing office spaces in Kansai Section and B-Cabin Road, Ambernath East. Assured rental yields up to 8% per annum with clear titles. Contact Satnam Sir for on-site inspection and customized investor deals.</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:31:05.356059</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792825261101</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>238+ Verified MMR Real Estate Projects &amp; Estates Directory Live [AI Verified: 24 Oct]</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Dashmesh Properties proudly unveils the largest verified MMR project directory covering 16 regional hubs: Ambernath (29 projects), Badlapur (17), Ulhasnagar (19), Kalyan (24), Dombivli (15), Thane (22), Navi Mumbai (24) and Mumbai. Check exact carpet areas, RERA numbers, and builder pricing.</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:31:05.357829</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(mrea-si): implement connected real-data super-intelligence multi-agent automation engine
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -776,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.685880</t>
+          <t>2026-10-25T16:17:30.863797</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.685898</t>
+          <t>2026-10-25T16:17:30.863811</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.685915</t>
+          <t>2026-10-25T16:17:30.863826</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.685864</t>
+          <t>2026-10-25T16:17:30.863782</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.685847</t>
+          <t>2026-10-25T16:17:30.863768</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.685829</t>
+          <t>2026-10-25T16:17:30.863753</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.685778</t>
+          <t>2026-10-25T16:17:30.863737</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,12 +1232,110 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.684056</t>
+          <t>2026-10-25T16:17:30.863718</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
           <t>2026-10-20T00:12:51.518788</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>+919137156440</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Skill Circle</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>New Inquiry</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Rent Agreement (₹1750/side)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Ambernath East</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>hinglish</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Inquiry</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:17:30.863654</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T14:25:00.436741</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>+918287617759</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>New Inquiry</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Rent Agreement (₹1750/side)</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Ambernath East</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>hinglish</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Inquiry</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:17:30.861052</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25T15:56:09.806301</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1475,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.694109</t>
+          <t>2026-10-25T16:17:30.875147</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1418,7 +1516,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.695302</t>
+          <t>2026-10-25T16:17:30.876654</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1459,7 +1557,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.695352</t>
+          <t>2026-10-25T16:17:30.876708</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1500,7 +1598,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.695373</t>
+          <t>2026-10-25T16:17:30.876727</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1541,7 +1639,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.695388</t>
+          <t>2026-10-25T16:17:30.876742</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1582,7 +1680,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.695402</t>
+          <t>2026-10-25T16:17:30.876756</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1623,7 +1721,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.695422</t>
+          <t>2026-10-25T16:17:30.876786</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1664,7 +1762,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T13:00:47.695438</t>
+          <t>2026-10-25T16:17:30.876800</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1695,7 +1793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2660,7 +2758,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -2693,7 +2791,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -2726,7 +2824,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -2759,7 +2857,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2796,7 +2894,7 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -2833,7 +2931,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2870,7 +2968,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2907,7 +3005,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2940,7 +3038,7 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -2977,7 +3075,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -3010,7 +3108,7 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -3047,7 +3145,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -3084,7 +3182,7 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
@@ -3121,7 +3219,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -3158,7 +3256,7 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -3195,7 +3293,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -3232,7 +3330,7 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
@@ -3269,7 +3367,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -3306,7 +3404,7 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -3343,7 +3441,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -3380,7 +3478,7 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -3417,7 +3515,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3454,7 +3552,7 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
@@ -3491,7 +3589,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3528,7 +3626,7 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
@@ -3565,7 +3663,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3602,7 +3700,7 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
@@ -3639,7 +3737,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3676,7 +3774,7 @@
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
@@ -3713,7 +3811,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -3750,7 +3848,7 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
@@ -3787,7 +3885,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -3861,7 +3959,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -3898,7 +3996,7 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
@@ -3935,7 +4033,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -3972,7 +4070,7 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
@@ -4009,7 +4107,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -4046,7 +4144,7 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
@@ -4083,7 +4181,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -4120,7 +4218,7 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
@@ -4231,7 +4329,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -4268,7 +4366,7 @@
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
@@ -4305,7 +4403,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -4342,7 +4440,7 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
@@ -4379,7 +4477,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -4412,7 +4510,7 @@
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
@@ -4449,7 +4547,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -4486,7 +4584,7 @@
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
@@ -4597,7 +4695,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -4634,7 +4732,7 @@
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
@@ -4671,7 +4769,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -4682,6 +4780,80 @@
       <c r="G82" s="2" t="inlineStr">
         <is>
           <t>2026-10-24T12:31:05.357829</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1792917849723</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 25 Oct]</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25T14:14:11.155503</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1792925221699</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 25 Oct]</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:17:03.178931</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: unified 4-channel cross-posting (Google, FB, Insta, LinkedIn) + SEO guardian + 24/7 loop engine
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -776,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -785,7 +785,7 @@
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.863797</t>
+          <t>2026-10-28T17:16:09.246573</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.863811</t>
+          <t>2026-10-28T17:16:09.246578</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.863826</t>
+          <t>2026-10-28T17:16:09.246583</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.863782</t>
+          <t>2026-10-28T17:16:09.246568</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.863768</t>
+          <t>2026-10-28T17:16:09.246562</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.863753</t>
+          <t>2026-10-28T17:16:09.246557</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.863737</t>
+          <t>2026-10-28T17:16:09.246552</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.863718</t>
+          <t>2026-10-28T17:16:09.246546</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1281,7 +1281,7 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.863654</t>
+          <t>2026-10-28T17:16:09.246523</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1330,12 +1330,61 @@
       <c r="I11" s="4" t="inlineStr"/>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.861052</t>
+          <t>2026-10-28T17:16:09.245612</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
           <t>2026-10-25T15:56:09.806301</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>+919988776655</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Rajesh Sharma ji</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>New Inquiry</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Rent Agreement (₹1750/side)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Ambernath East</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Hindi / English</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Inquiry</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T21:19:05.103653</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T21:05:18.434760</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1524,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.875147</t>
+          <t>2026-10-28T17:16:09.267842</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1516,7 +1565,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.876654</t>
+          <t>2026-10-28T17:16:09.268646</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1557,7 +1606,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.876708</t>
+          <t>2026-10-28T17:16:09.268667</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1598,7 +1647,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.876727</t>
+          <t>2026-10-28T17:16:09.268672</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1639,7 +1688,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.876742</t>
+          <t>2026-10-28T17:16:09.268677</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1680,7 +1729,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.876756</t>
+          <t>2026-10-28T17:16:09.268682</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1721,7 +1770,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.876786</t>
+          <t>2026-10-28T17:16:09.268689</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1762,7 +1811,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25T16:17:30.876800</t>
+          <t>2026-10-28T17:16:09.268693</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1793,15 +1842,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="33" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="31" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2824,7 +2873,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -2857,7 +2906,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2894,7 +2943,7 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -2931,7 +2980,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2968,7 +3017,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -3005,7 +3054,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -3038,7 +3087,7 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -3075,7 +3124,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -3108,7 +3157,7 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -3145,7 +3194,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -3182,7 +3231,7 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
@@ -3219,7 +3268,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -3256,7 +3305,7 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -3293,7 +3342,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -3330,7 +3379,7 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
@@ -3367,7 +3416,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -3404,7 +3453,7 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -3441,7 +3490,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -3478,7 +3527,7 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -3515,7 +3564,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3552,7 +3601,7 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
@@ -3589,7 +3638,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3626,7 +3675,7 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
@@ -3663,7 +3712,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3700,7 +3749,7 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
@@ -3737,7 +3786,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3774,7 +3823,7 @@
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
@@ -3811,7 +3860,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -3848,7 +3897,7 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
@@ -3885,7 +3934,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -3959,7 +4008,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -3996,7 +4045,7 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
@@ -4033,7 +4082,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -4070,7 +4119,7 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
@@ -4107,7 +4156,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -4144,7 +4193,7 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
@@ -4181,7 +4230,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -4218,7 +4267,7 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
@@ -4329,7 +4378,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -4366,7 +4415,7 @@
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
@@ -4403,7 +4452,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -4440,7 +4489,7 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
@@ -4477,7 +4526,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -4510,7 +4559,7 @@
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
@@ -4547,7 +4596,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -4584,7 +4633,7 @@
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
@@ -4695,7 +4744,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -4732,7 +4781,7 @@
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
@@ -4769,7 +4818,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -4806,7 +4855,7 @@
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
@@ -4843,7 +4892,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -4854,6 +4903,257 @@
       <c r="G84" s="2" t="inlineStr">
         <is>
           <t>2026-10-25T16:17:03.178931</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1793028851362</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 26 Oct]</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-26T21:04:12.782793</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1793184413557</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 28 Oct]</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28T16:16:55.166739</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1793185892649</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>1 BHK &amp; 2 BHK Affordable Luxury Flats in Pale Gaon, Ambernath East [AI Verified: 28 Oct]</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Discover verified ready-to-move and under-construction flats starting ₹19.5 Lakhs in prime Pale Gaon and Shiv Mandir Road. SBI &amp; HDFC pre-approved up to 90% loan, KDMC water, 5 mins from Ambernath East station. Zero brokerage deals available directly via Dashmesh Properties.</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-28T16:41:34.522803</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1793186248056</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>238+ Verified MMR Real Estate Projects &amp; Estates Directory Live [AI Verified: 28 Oct]</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Dashmesh Properties proudly unveils the largest verified MMR project directory covering 16 regional hubs: Ambernath (29 projects), Badlapur (17), Ulhasnagar (19), Kalyan (24), Dombivli (15), Thane (22), Navi Mumbai (24) and Mumbai. Check exact carpet areas, RERA numbers, and builder pricing.</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28T16:47:29.581529</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1793187344825</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 28 Oct]</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-28T17:05:46.347857</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>omni_broadcast_1793187366926</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Navratri Special 1 BHK Flats in Pale Gaon</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr"/>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>CALL_NOW</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Omni-Broadcast Complete (4/4 Channels Live)</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28T17:09:08.789628</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>omni_broadcast_1793187818104</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Laxmi Niwas Pale Gaon 2 BHK Luxury Balcony</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr"/>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>CALL_NOW</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>Omni-Broadcast Complete (4/4 Channels Live)</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-28T17:16:09.232816</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): enforce strict zero fake leads policy & persist clean verified records
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.321597</t>
+          <t>2026-10-28T22:59:17.907307</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.321608</t>
+          <t>2026-10-28T22:59:17.907312</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.321618</t>
+          <t>2026-10-28T22:59:17.907317</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.321587</t>
+          <t>2026-10-28T22:59:17.907302</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.321576</t>
+          <t>2026-10-28T22:59:17.907297</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.321563</t>
+          <t>2026-10-28T22:59:17.907291</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1281,7 +1281,7 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.321523</t>
+          <t>2026-10-28T22:59:17.907274</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1330,7 +1330,7 @@
       <c r="I11" s="4" t="inlineStr"/>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.319933</t>
+          <t>2026-10-28T22:59:17.906628</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.345638</t>
+          <t>2026-10-28T22:59:17.913900</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.348489</t>
+          <t>2026-10-28T22:59:17.914950</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.348541</t>
+          <t>2026-10-28T22:59:17.914990</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.348557</t>
+          <t>2026-10-28T22:59:17.914998</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.348571</t>
+          <t>2026-10-28T22:59:17.915004</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.348583</t>
+          <t>2026-10-28T22:59:17.915009</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.348601</t>
+          <t>2026-10-28T22:59:17.915018</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:54:03.348613</t>
+          <t>2026-10-28T22:59:17.915023</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1842,7 +1842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5191,6 +5191,80 @@
       <c r="G92" s="2" t="inlineStr">
         <is>
           <t>2026-10-28T21:02:58.038864</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1793208556411</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 28 Oct]</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-28T22:59:17.922179</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1793208469670</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 28 Oct]</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28T22:59:17.923381</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(whatsapp): revamp WhatsApp AI conversational engine with zero repetitive greetings and Chief-of-Staff capabilities
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -776,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.907307</t>
+          <t>2026-10-29T01:23:10.360759</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.907312</t>
+          <t>2026-10-29T01:23:10.360767</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.907317</t>
+          <t>2026-10-29T01:23:10.360774</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.907302</t>
+          <t>2026-10-29T01:23:10.360751</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.907297</t>
+          <t>2026-10-29T01:23:10.360743</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.907291</t>
+          <t>2026-10-29T01:23:10.360734</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1281,7 +1281,7 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.907274</t>
+          <t>2026-10-29T01:23:10.360724</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1330,7 +1330,7 @@
       <c r="I11" s="4" t="inlineStr"/>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.906628</t>
+          <t>2026-10-29T01:23:10.360687</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
@@ -1385,6 +1385,55 @@
       <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-10-26T21:05:18.434760</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>+916260347690</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>VIKASH</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>New Inquiry</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Rent Agreement (₹1750/side)</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr"/>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Ambernath East</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>hinglish</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Inquiry</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29T01:23:10.359424</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29T00:31:28.211320</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1573,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.913900</t>
+          <t>2026-10-29T01:23:10.368454</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1565,7 +1614,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.914950</t>
+          <t>2026-10-29T01:23:10.369530</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1606,7 +1655,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.914990</t>
+          <t>2026-10-29T01:23:10.369579</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1647,7 +1696,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.914998</t>
+          <t>2026-10-29T01:23:10.369588</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1688,7 +1737,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.915004</t>
+          <t>2026-10-29T01:23:10.369596</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1729,7 +1778,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.915009</t>
+          <t>2026-10-29T01:23:10.369604</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1770,7 +1819,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.915018</t>
+          <t>2026-10-29T01:23:10.369616</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1811,7 +1860,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T22:59:17.915023</t>
+          <t>2026-10-29T01:23:10.369623</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1842,7 +1891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3305,7 +3354,7 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -3342,7 +3391,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -3379,7 +3428,7 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
@@ -3416,7 +3465,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -3453,7 +3502,7 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -3490,7 +3539,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -3527,7 +3576,7 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -3564,7 +3613,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3601,7 +3650,7 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
@@ -3638,7 +3687,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3675,7 +3724,7 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
@@ -3712,7 +3761,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3749,7 +3798,7 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
@@ -3786,7 +3835,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3823,7 +3872,7 @@
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
@@ -3860,7 +3909,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -3897,7 +3946,7 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
@@ -3934,7 +3983,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -4008,7 +4057,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -4045,7 +4094,7 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
@@ -4082,7 +4131,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -4119,7 +4168,7 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
@@ -4156,7 +4205,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -4193,7 +4242,7 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
@@ -4230,7 +4279,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -4267,7 +4316,7 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
@@ -4378,7 +4427,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -4415,7 +4464,7 @@
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
@@ -4452,7 +4501,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -4489,7 +4538,7 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
@@ -4526,7 +4575,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -4559,7 +4608,7 @@
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
@@ -4596,7 +4645,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -4633,7 +4682,7 @@
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
@@ -4744,7 +4793,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -4781,7 +4830,7 @@
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
@@ -4818,7 +4867,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -4855,7 +4904,7 @@
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
@@ -4892,7 +4941,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -4929,7 +4978,7 @@
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
@@ -4966,7 +5015,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -5003,7 +5052,7 @@
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
@@ -5040,7 +5089,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -5077,7 +5126,7 @@
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
@@ -5110,7 +5159,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -5143,7 +5192,7 @@
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr">
@@ -5180,7 +5229,7 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -5217,7 +5266,7 @@
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F93" s="4" t="inlineStr">
@@ -5254,7 +5303,7 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -5265,6 +5314,117 @@
       <c r="G94" s="2" t="inlineStr">
         <is>
           <t>2026-10-28T22:59:17.923381</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1793210288296</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 28 Oct]</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="F95" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-28T23:28:10.191584</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1793214187903</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 29 Oct]</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29T00:33:09.820916</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>aipost_1793217093025</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 29 Oct]</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29T01:21:34.839230</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(whatsapp-ai): eliminate greeting loop, answer complete compound questions, and persist conversation memory across restarts
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.360759</t>
+          <t>2026-10-30T00:47:46.830099</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.360767</t>
+          <t>2026-10-30T00:47:46.830109</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.360774</t>
+          <t>2026-10-30T00:47:46.830116</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.360751</t>
+          <t>2026-10-30T00:47:46.830089</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.360743</t>
+          <t>2026-10-30T00:47:46.830081</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.360734</t>
+          <t>2026-10-30T00:47:46.830072</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1281,7 +1281,7 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.360724</t>
+          <t>2026-10-30T00:47:46.830062</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1330,7 +1330,7 @@
       <c r="I11" s="4" t="inlineStr"/>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.360687</t>
+          <t>2026-10-30T00:47:46.829998</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
@@ -1428,7 +1428,7 @@
       <c r="I13" s="4" t="inlineStr"/>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.359424</t>
+          <t>2026-10-30T00:47:46.828244</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.368454</t>
+          <t>2026-10-30T00:47:46.931635</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.369530</t>
+          <t>2026-10-30T00:47:46.933897</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.369579</t>
+          <t>2026-10-30T00:47:46.933943</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.369588</t>
+          <t>2026-10-30T00:47:46.933950</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.369596</t>
+          <t>2026-10-30T00:47:46.933955</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.369604</t>
+          <t>2026-10-30T00:47:46.933961</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.369616</t>
+          <t>2026-10-30T00:47:46.933972</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T01:23:10.369623</t>
+          <t>2026-10-30T00:47:46.933977</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1891,7 +1891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G97"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3465,7 +3465,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -3502,7 +3502,7 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -3539,7 +3539,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -3613,7 +3613,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
@@ -3687,7 +3687,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3724,7 +3724,7 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
@@ -3835,7 +3835,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3872,7 +3872,7 @@
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
@@ -3909,7 +3909,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -3946,7 +3946,7 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -4094,7 +4094,7 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -4168,7 +4168,7 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
@@ -4205,7 +4205,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -4242,7 +4242,7 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
@@ -4279,7 +4279,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -4316,7 +4316,7 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
@@ -4501,7 +4501,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -4538,7 +4538,7 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
@@ -4645,7 +4645,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -4682,7 +4682,7 @@
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
@@ -4793,7 +4793,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -4830,7 +4830,7 @@
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
@@ -4867,7 +4867,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -4904,7 +4904,7 @@
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -4978,7 +4978,7 @@
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
@@ -5015,7 +5015,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
@@ -5089,7 +5089,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
@@ -5159,7 +5159,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -5192,7 +5192,7 @@
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr">
@@ -5229,7 +5229,7 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -5266,7 +5266,7 @@
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F93" s="4" t="inlineStr">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -5340,7 +5340,7 @@
       </c>
       <c r="E95" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F95" s="4" t="inlineStr">
@@ -5377,7 +5377,7 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F97" s="4" t="inlineStr">
@@ -5425,6 +5425,43 @@
       <c r="G97" s="4" t="inlineStr">
         <is>
           <t>2026-10-29T01:21:34.839230</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>aipost_1793300419006</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Official Registered Rent Agreement at ₹1,750 (Doorstep Biometric) [AI Verified: 30 Oct]</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Need Govt Registered Rent Agreement in Ambernath, Badlapur, Ulhasnagar or Kalyan? Dashmesh Properties provides 100% legal e-registration with doorstep biometric verification for just ₹1,750 per side (₹3,500 all-inclusive with stamp duty &amp; registration). Instant slot booking!</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Book Doorstep Biometric (+91 84210 77613)</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Published (AI Autonomous)</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30T00:30:21.174733</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(deploy): resolve Render launch failures with dynamic PORT binding, multi-port healthcheck, Node 20 engines, and package-lock
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.830099</t>
+          <t>2026-10-30T01:29:59.410473</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.830109</t>
+          <t>2026-10-30T01:29:59.410478</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.830116</t>
+          <t>2026-10-30T01:29:59.410483</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.830089</t>
+          <t>2026-10-30T01:29:59.410468</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.830081</t>
+          <t>2026-10-30T01:29:59.410462</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.830072</t>
+          <t>2026-10-30T01:29:59.410457</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1281,7 +1281,7 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.830062</t>
+          <t>2026-10-30T01:29:59.410450</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1330,7 +1330,7 @@
       <c r="I11" s="4" t="inlineStr"/>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.829998</t>
+          <t>2026-10-30T01:29:59.410423</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
@@ -1428,7 +1428,7 @@
       <c r="I13" s="4" t="inlineStr"/>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.828244</t>
+          <t>2026-10-30T01:29:59.409430</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.931635</t>
+          <t>2026-10-30T01:29:59.417302</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.933897</t>
+          <t>2026-10-30T01:29:59.418197</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.933943</t>
+          <t>2026-10-30T01:29:59.418221</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.933950</t>
+          <t>2026-10-30T01:29:59.418227</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.933955</t>
+          <t>2026-10-30T01:29:59.418232</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.933961</t>
+          <t>2026-10-30T01:29:59.418237</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.933972</t>
+          <t>2026-10-30T01:29:59.418244</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T00:47:46.933977</t>
+          <t>2026-10-30T01:29:59.418249</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: sync latest runtime config and database snapshot
</commit_message>
<xml_diff>
--- a/data/Dashmesh_Master_Database.xlsx
+++ b/data/Dashmesh_Master_Database.xlsx
@@ -889,7 +889,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.410473</t>
+          <t>2026-10-30T01:44:02.222375</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="I3" s="4" t="inlineStr"/>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.410478</t>
+          <t>2026-10-30T01:44:02.222380</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.410483</t>
+          <t>2026-10-30T01:44:02.222385</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.410468</t>
+          <t>2026-10-30T01:44:02.222370</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.410462</t>
+          <t>2026-10-30T01:44:02.222365</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.410457</t>
+          <t>2026-10-30T01:44:02.222360</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1281,7 +1281,7 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.410450</t>
+          <t>2026-10-30T01:44:02.222354</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1330,7 +1330,7 @@
       <c r="I11" s="4" t="inlineStr"/>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.410423</t>
+          <t>2026-10-30T01:44:02.222320</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
@@ -1428,7 +1428,7 @@
       <c r="I13" s="4" t="inlineStr"/>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.409430</t>
+          <t>2026-10-30T01:44:02.221370</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.417302</t>
+          <t>2026-10-30T01:44:02.246216</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.418197</t>
+          <t>2026-10-30T01:44:02.246917</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.418221</t>
+          <t>2026-10-30T01:44:02.246936</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.418227</t>
+          <t>2026-10-30T01:44:02.246942</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.418232</t>
+          <t>2026-10-30T01:44:02.246947</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.418237</t>
+          <t>2026-10-30T01:44:02.246951</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.418244</t>
+          <t>2026-10-30T01:44:02.246958</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:29:59.418249</t>
+          <t>2026-10-30T01:44:02.246962</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">

</xml_diff>